<commit_message>
Align ATR and historical windows with market periods
</commit_message>
<xml_diff>
--- a/tokenDemo/close_records.xlsx
+++ b/tokenDemo/close_records.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M11"/>
+  <dimension ref="A1:M12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -993,6 +993,57 @@
       </c>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-09-01 14:37:02</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>潞化科技 600691</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>3.23</v>
+      </c>
+      <c r="E12" t="n">
+        <v>3.35</v>
+      </c>
+      <c r="F12" t="n">
+        <v>100</v>
+      </c>
+      <c r="G12" t="n">
+        <v>12.00000000000001</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>3.72%</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>100.00%</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>BZ</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>首次止盈</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1005,7 +1056,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M560"/>
+  <dimension ref="A1:M561"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27378,6 +27429,65 @@
         </is>
       </c>
     </row>
+    <row r="561">
+      <c r="A561" t="inlineStr">
+        <is>
+          <t>2026-09-01 15:03:02</t>
+        </is>
+      </c>
+      <c r="B561" t="inlineStr">
+        <is>
+          <t>AGTUSDT</t>
+        </is>
+      </c>
+      <c r="C561" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D561" t="n">
+        <v>0.01762783449924071</v>
+      </c>
+      <c r="E561" t="n">
+        <v>0.015668</v>
+      </c>
+      <c r="F561" t="n">
+        <v>40169</v>
+      </c>
+      <c r="G561" t="n">
+        <v>-78.72459199999987</v>
+      </c>
+      <c r="H561" t="inlineStr">
+        <is>
+          <t>-11.12%</t>
+        </is>
+      </c>
+      <c r="I561" t="inlineStr">
+        <is>
+          <t>100.00%</t>
+        </is>
+      </c>
+      <c r="J561" t="inlineStr">
+        <is>
+          <t>BZ,DCA*2</t>
+        </is>
+      </c>
+      <c r="K561" t="inlineStr">
+        <is>
+          <t>移动止损(轨道)</t>
+        </is>
+      </c>
+      <c r="L561" t="inlineStr">
+        <is>
+          <t>1.5458</t>
+        </is>
+      </c>
+      <c r="M561" t="inlineStr">
+        <is>
+          <t>0.2979%</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>